<commit_message>
Batch 3: 10 parent and school-start videos, 2 new themes
- Themes: paper (paper-cut), sunrise (dawn gradient)
- Episodes K3 K4 K6 K7 K8 I6 I4 F6 I7 E6, silent + AI-voiced cuts
- Topic workbook updated to 68 topics with batch-3 status
- docs: batch-3 notes with sources and release timing

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q1wfgpLC9KuF9JDcMQwYSx
</commit_message>
<xml_diff>
--- a/docs/视频主题清单.xlsx
+++ b/docs/视频主题清单.xlsx
@@ -13,7 +13,7 @@
     <sheet name="说明" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">主题清单!$A$1:$N$62</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">主题清单!$A$1:$N$69</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="429">
   <si>
     <t xml:space="preserve">类型</t>
   </si>
@@ -4719,6 +4719,176 @@
     <t xml:space="preserve">做减法，是最快的加法</t>
   </si>
   <si>
+    <t xml:space="preserve">E6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">学习时，手机放哪？</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Ward </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">等（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2017</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）近 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">800 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">人实验：手机放在另一个房间的人测试表现最好，放桌上最差，即使静音朝下</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">学习的时候，让手机离开房间</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">批</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">号男声</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">E6_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">学习时手机放哪</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">无配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 / _AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">F1</t>
   </si>
   <si>
@@ -5162,25 +5332,6 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">号男声</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
       <t xml:space="preserve">F2_</t>
     </r>
     <r>
@@ -5336,6 +5487,181 @@
     <t xml:space="preserve">错题不是失败，是你的梯度</t>
   </si>
   <si>
+    <t xml:space="preserve">F6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">新学期目标，拆小了才能完成</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Bandura &amp; Schunk</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1981</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">42 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">页数学练习，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每次 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">页</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">的小目标组进步最快、最有信心</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">大目标定方向，小目标给动力</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">F6_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">新学期目标拆小了才能完成</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">无配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 / _AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">G1</t>
   </si>
   <si>
@@ -6452,6 +6778,85 @@
     <t xml:space="preserve">高三</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">I4_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">最后</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">无配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 / _AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">I5</t>
   </si>
   <si>
@@ -6488,6 +6893,357 @@
     <t xml:space="preserve">每个阶段，都有它该做的事</t>
   </si>
   <si>
+    <t xml:space="preserve">I6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">开学前，先把生物钟拨回来</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">寒假与上学作息差 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小时；倒时差经验每天约调 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小时 → 至少提前 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天开始</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">先把生物钟，拨回开学模式</t>
+  </si>
+  <si>
+    <t xml:space="preserve">晨光</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">I6_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">开学前先把生物钟拨回来</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">无配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 / _AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">I7</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">新学期，其实只有 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">周</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">周 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× 5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= 90 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天课；第 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">9 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">周期中；晚 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">周进入状态就少 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">周</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">新学期，从第一周开始算数</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">I7_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">新学期其实只有</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">周</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">无配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 / _AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">J1</t>
   </si>
   <si>
@@ -7182,16 +7938,167 @@
     <t xml:space="preserve">支持要和孩子同频，才有用</t>
   </si>
   <si>
+    <t xml:space="preserve">纸雕</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">K3_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">同频才能放大</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">无配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 / _AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">K4</t>
   </si>
   <si>
-    <t xml:space="preserve">风筝的线</t>
-  </si>
-  <si>
-    <t xml:space="preserve">风筝受力分析：线太紧会断，太松会坠</t>
-  </si>
-  <si>
-    <t xml:space="preserve">托举，不是攥紧</t>
+    <t xml:space="preserve">别把孩子的弹簧拉坏了</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">胡克定律 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">F = kx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（弹性限度内）；超过弹性限度发生塑性形变，撤去外力回不到原长</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">给压力，也要给孩子留弹性</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">K4_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">别把孩子的弹簧拉坏了</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">无配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 / _AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">K5</t>
@@ -7206,6 +8113,363 @@
     <t xml:space="preserve">选对帮助，比给更多帮助重要</t>
   </si>
   <si>
+    <t xml:space="preserve">K6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">孩子每天该睡几个小时？</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">教育部（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2021</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）：高中生每天睡眠应达 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小时；只睡 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小时一周欠 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小时；睡眠中记忆巩固</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">睡够了，学进去的才留得住</t>
+  </si>
+  <si>
+    <t xml:space="preserve">流光渐变</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">K6_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">孩子每天该睡几个小时</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">无配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 / _AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">K7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">夸孩子聪明，还是夸努力？</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Mueller &amp; Dweck</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1998</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）：被夸聪明的孩子更多选简单题、受挫易放弃；被夸努力的更多选难题</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">少夸你真聪明，多夸你真努力</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">K7_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">夸孩子聪明还是夸努力</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">无配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 / _AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">K8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">孩子不听你说什么，看你做什么</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">班杜拉波波玩偶实验（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1961</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）：儿童模仿成人行为（观察学习）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">最好的教育，是做给孩子看</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">K8_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">孩子看你做什么</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">无配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4 / _AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">配音</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.mp4</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">L1</t>
   </si>
   <si>
@@ -7262,9 +8526,6 @@
     <t xml:space="preserve">考前学生</t>
   </si>
   <si>
-    <t xml:space="preserve">流光渐变</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="10"/>
@@ -7633,6 +8894,23 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">68 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">个主题（原规划 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">61 </t>
     </r>
     <r>
@@ -7641,7 +8919,75 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">个主题。每个主题都以一个真实的科学事实或算出来的数字作锚点，前 </t>
+      <t xml:space="preserve">个 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">第 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">批新增 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">个，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">K4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">换题）。每个主题都以一个真实的科学事实或算出来的数字作锚点，前 </t>
     </r>
     <r>
       <rPr>
@@ -8737,11 +10083,11 @@
         <v>12</v>
       </c>
       <c r="F2" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A2)</f>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A2)</f>
         <v>6</v>
       </c>
       <c r="G2" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A2,主题清单!$J$2:$J$62,"已制作")</f>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A2,主题清单!$J$2:$J$69,"已制作")</f>
         <v>2</v>
       </c>
       <c r="H2" s="2" t="n">
@@ -8766,11 +10112,11 @@
         <v>17</v>
       </c>
       <c r="F3" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A3)</f>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A3)</f>
         <v>6</v>
       </c>
       <c r="G3" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A3,主题清单!$J$2:$J$62,"已制作")</f>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A3,主题清单!$J$2:$J$69,"已制作")</f>
         <v>2</v>
       </c>
       <c r="H3" s="2" t="n">
@@ -8795,11 +10141,11 @@
         <v>21</v>
       </c>
       <c r="F4" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A4)</f>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A4)</f>
         <v>6</v>
       </c>
       <c r="G4" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A4,主题清单!$J$2:$J$62,"已制作")</f>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A4,主题清单!$J$2:$J$69,"已制作")</f>
         <v>4</v>
       </c>
       <c r="H4" s="2" t="n">
@@ -8824,11 +10170,11 @@
         <v>24</v>
       </c>
       <c r="F5" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A5)</f>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A5)</f>
         <v>5</v>
       </c>
       <c r="G5" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A5,主题清单!$J$2:$J$62,"已制作")</f>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A5,主题清单!$J$2:$J$69,"已制作")</f>
         <v>1</v>
       </c>
       <c r="H5" s="2" t="n">
@@ -8853,12 +10199,12 @@
         <v>28</v>
       </c>
       <c r="F6" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A6)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A6)</f>
+        <v>6</v>
       </c>
       <c r="G6" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A6,主题清单!$J$2:$J$62,"已制作")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A6,主题清单!$J$2:$J$69,"已制作")</f>
+        <v>2</v>
       </c>
       <c r="H6" s="2" t="n">
         <f aca="false">F6-G6</f>
@@ -8882,12 +10228,12 @@
         <v>32</v>
       </c>
       <c r="F7" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A7)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A7)</f>
+        <v>6</v>
       </c>
       <c r="G7" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A7,主题清单!$J$2:$J$62,"已制作")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A7,主题清单!$J$2:$J$69,"已制作")</f>
+        <v>3</v>
       </c>
       <c r="H7" s="2" t="n">
         <f aca="false">F7-G7</f>
@@ -8911,11 +10257,11 @@
         <v>35</v>
       </c>
       <c r="F8" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A8)</f>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A8)</f>
         <v>5</v>
       </c>
       <c r="G8" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A8,主题清单!$J$2:$J$62,"已制作")</f>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A8,主题清单!$J$2:$J$69,"已制作")</f>
         <v>3</v>
       </c>
       <c r="H8" s="2" t="n">
@@ -8940,11 +10286,11 @@
         <v>38</v>
       </c>
       <c r="F9" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A9)</f>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A9)</f>
         <v>4</v>
       </c>
       <c r="G9" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A9,主题清单!$J$2:$J$62,"已制作")</f>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A9,主题清单!$J$2:$J$69,"已制作")</f>
         <v>1</v>
       </c>
       <c r="H9" s="2" t="n">
@@ -8969,16 +10315,16 @@
         <v>41</v>
       </c>
       <c r="F10" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A10)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A10)</f>
+        <v>7</v>
       </c>
       <c r="G10" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A10,主题清单!$J$2:$J$62,"已制作")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A10,主题清单!$J$2:$J$69,"已制作")</f>
+        <v>4</v>
       </c>
       <c r="H10" s="2" t="n">
         <f aca="false">F10-G10</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8998,11 +10344,11 @@
         <v>45</v>
       </c>
       <c r="F11" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A11)</f>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A11)</f>
         <v>5</v>
       </c>
       <c r="G11" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A11,主题清单!$J$2:$J$62,"已制作")</f>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A11,主题清单!$J$2:$J$69,"已制作")</f>
         <v>2</v>
       </c>
       <c r="H11" s="2" t="n">
@@ -9027,16 +10373,16 @@
         <v>49</v>
       </c>
       <c r="F12" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A12)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A12)</f>
+        <v>8</v>
       </c>
       <c r="G12" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A12,主题清单!$J$2:$J$62,"已制作")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A12,主题清单!$J$2:$J$69,"已制作")</f>
+        <v>7</v>
       </c>
       <c r="H12" s="2" t="n">
         <f aca="false">F12-G12</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9056,11 +10402,11 @@
         <v>53</v>
       </c>
       <c r="F13" s="2" t="n">
-        <f aca="false">COUNTIF(主题清单!$B$2:$B$62,A13)</f>
+        <f aca="false">COUNTIF(主题清单!$B$2:$B$69,A13)</f>
         <v>4</v>
       </c>
       <c r="G13" s="2" t="n">
-        <f aca="false">COUNTIFS(主题清单!$B$2:$B$62,A13,主题清单!$J$2:$J$62,"已制作")</f>
+        <f aca="false">COUNTIFS(主题清单!$B$2:$B$69,A13,主题清单!$J$2:$J$69,"已制作")</f>
         <v>2</v>
       </c>
       <c r="H13" s="2" t="n">
@@ -9074,15 +10420,15 @@
       </c>
       <c r="F14" s="8" t="n">
         <f aca="false">SUM(F2:F13)</f>
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="G14" s="8" t="n">
         <f aca="false">SUM(G2:G13)</f>
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="H14" s="8" t="n">
         <f aca="false">SUM(H2:H13)</f>
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9091,7 +10437,7 @@
       </c>
       <c r="G15" s="9" t="n">
         <f aca="false">IF(F14=0,0,G14/F14)</f>
-        <v>0.377049180327869</v>
+        <v>0.485294117647059</v>
       </c>
     </row>
   </sheetData>
@@ -9110,7 +10456,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N62"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -10229,7 +11575,7 @@
         <v>215</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>26</v>
@@ -10237,7 +11583,7 @@
       <c r="D30" s="11" t="s">
         <v>216</v>
       </c>
-      <c r="E30" s="11" t="s">
+      <c r="E30" s="10" t="s">
         <v>217</v>
       </c>
       <c r="F30" s="11" t="s">
@@ -10249,17 +11595,15 @@
       <c r="H30" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="I30" s="10" t="s">
-        <v>74</v>
-      </c>
+      <c r="I30" s="10"/>
       <c r="J30" s="11" t="s">
         <v>6</v>
       </c>
       <c r="K30" s="11" t="s">
-        <v>75</v>
+        <v>219</v>
       </c>
       <c r="L30" s="11" t="s">
-        <v>219</v>
+        <v>76</v>
       </c>
       <c r="M30" s="10" t="s">
         <v>220</v>
@@ -10303,52 +11647,62 @@
         <v>75</v>
       </c>
       <c r="L31" s="11" t="s">
-        <v>110</v>
+        <v>226</v>
       </c>
       <c r="M31" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="B32" s="2" t="s">
+      <c r="A32" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="B32" s="10" t="s">
         <v>29</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D32" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="E32" s="4" t="s">
+      <c r="D32" s="11" t="s">
         <v>230</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="E32" s="11" t="s">
         <v>231</v>
       </c>
-      <c r="G32" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="I32" s="2"/>
-      <c r="J32" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
-      <c r="N32" s="2"/>
+      <c r="F32" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G32" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I32" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J32" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K32" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="L32" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="M32" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="N32" s="10" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>29</v>
@@ -10357,19 +11711,19 @@
         <v>26</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="4" t="s">
@@ -10382,7 +11736,7 @@
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>29</v>
@@ -10390,17 +11744,17 @@
       <c r="C34" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>237</v>
+      <c r="D34" s="4" t="s">
+        <v>239</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>20</v>
+        <v>83</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>73</v>
@@ -10415,231 +11769,229 @@
       <c r="N34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D35" s="10" t="s">
-        <v>241</v>
-      </c>
-      <c r="E35" s="11" t="s">
+      <c r="A35" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="F35" s="11" t="s">
+      <c r="B35" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="G35" s="11" t="s">
+      <c r="E35" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="H35" s="10" t="s">
+      <c r="F35" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H35" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="I35" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="J35" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="K35" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="L35" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="M35" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="N35" s="10" t="s">
-        <v>245</v>
-      </c>
+      <c r="I35" s="2"/>
+      <c r="J35" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
         <v>246</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>9</v>
+        <v>29</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="D36" s="11" t="s">
         <v>247</v>
       </c>
-      <c r="E36" s="11" t="s">
+      <c r="E36" s="10" t="s">
         <v>248</v>
       </c>
       <c r="F36" s="11" t="s">
         <v>249</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="H36" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="I36" s="10" t="s">
-        <v>74</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="I36" s="10"/>
       <c r="J36" s="11" t="s">
         <v>6</v>
       </c>
       <c r="K36" s="11" t="s">
-        <v>109</v>
+        <v>219</v>
       </c>
       <c r="L36" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="M36" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="N36" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="M36" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="N36" s="10" t="s">
+    </row>
+    <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="10" t="s">
         <v>33</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="F37" s="11" t="s">
         <v>254</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="G37" s="11" t="s">
         <v>255</v>
       </c>
-      <c r="G37" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="H37" s="2" t="s">
+      <c r="H37" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="I37" s="2"/>
-      <c r="J37" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
-      <c r="N37" s="2"/>
+      <c r="I37" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J37" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K37" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="L37" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="M37" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="N37" s="10" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="B38" s="2" t="s">
+      <c r="A38" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="B38" s="10" t="s">
         <v>33</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D38" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="E38" s="4" t="s">
+      <c r="D38" s="11" t="s">
         <v>258</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="E38" s="11" t="s">
         <v>259</v>
       </c>
-      <c r="G38" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H38" s="2" t="s">
+      <c r="F38" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="G38" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="H38" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="I38" s="2"/>
-      <c r="J38" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
-      <c r="N38" s="2"/>
+      <c r="I38" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J38" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K38" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="L38" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="M38" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="N38" s="10" t="s">
+        <v>262</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="10" t="s">
-        <v>260</v>
-      </c>
-      <c r="B39" s="10" t="s">
+      <c r="A39" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>33</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D39" s="11" t="s">
-        <v>261</v>
-      </c>
-      <c r="E39" s="11" t="s">
-        <v>262</v>
-      </c>
-      <c r="F39" s="11" t="s">
-        <v>263</v>
-      </c>
-      <c r="G39" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="H39" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="I39" s="10"/>
-      <c r="J39" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="K39" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="L39" s="11" t="s">
+      <c r="D39" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="M39" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="N39" s="10" t="s">
+      <c r="E39" s="2" t="s">
         <v>265</v>
       </c>
+      <c r="F39" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="I39" s="2"/>
+      <c r="J39" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K39" s="2"/>
+      <c r="L39" s="2"/>
+      <c r="M39" s="2"/>
+      <c r="N39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="F40" s="4" t="s">
         <v>269</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>270</v>
       </c>
       <c r="G40" s="4" t="s">
         <v>48</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>74</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="I40" s="2"/>
       <c r="J40" s="4" t="s">
         <v>7</v>
       </c>
@@ -10648,53 +12000,51 @@
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
     </row>
-    <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G41" s="11" t="s">
         <v>201</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="I41" s="10" t="s">
-        <v>74</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="I41" s="10"/>
       <c r="J41" s="11" t="s">
         <v>6</v>
       </c>
       <c r="K41" s="11" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="L41" s="11" t="s">
-        <v>162</v>
+        <v>275</v>
       </c>
       <c r="M41" s="10" t="s">
-        <v>152</v>
+        <v>220</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>36</v>
@@ -10703,21 +12053,23 @@
         <v>9</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G42" s="4" t="s">
         <v>48</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="I42" s="2"/>
+        <v>73</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>74</v>
+      </c>
       <c r="J42" s="4" t="s">
         <v>7</v>
       </c>
@@ -10726,108 +12078,108 @@
       <c r="M42" s="2"/>
       <c r="N42" s="2"/>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="B43" s="2" t="s">
+    <row r="43" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="B43" s="10" t="s">
         <v>36</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D43" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="F43" s="4" t="s">
+      <c r="D43" s="11" t="s">
         <v>282</v>
       </c>
-      <c r="G43" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="I43" s="2"/>
-      <c r="J43" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K43" s="2"/>
-      <c r="L43" s="2"/>
-      <c r="M43" s="2"/>
-      <c r="N43" s="2"/>
+      <c r="E43" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="F43" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="G43" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I43" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J43" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K43" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="L43" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="M43" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="N43" s="10" t="s">
+        <v>285</v>
+      </c>
     </row>
-    <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="10" t="s">
-        <v>283</v>
-      </c>
-      <c r="B44" s="10" t="s">
-        <v>39</v>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D44" s="11" t="s">
-        <v>284</v>
-      </c>
-      <c r="E44" s="11" t="s">
-        <v>285</v>
-      </c>
-      <c r="F44" s="11" t="s">
-        <v>286</v>
-      </c>
-      <c r="G44" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="H44" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="I44" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="J44" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="K44" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="L44" s="11" t="s">
+      <c r="D44" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="M44" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="N44" s="10" t="s">
+      <c r="E44" s="4" t="s">
         <v>288</v>
       </c>
+      <c r="F44" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I44" s="2"/>
+      <c r="J44" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
+      <c r="N44" s="2"/>
     </row>
-    <row r="45" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>293</v>
+        <v>20</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="I45" s="2"/>
       <c r="J45" s="4" t="s">
@@ -10838,43 +12190,53 @@
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="2" t="s">
+    <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="10" t="s">
         <v>39</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D46" s="4" t="s">
+      <c r="D46" s="11" t="s">
         <v>295</v>
       </c>
-      <c r="E46" s="4" t="s">
+      <c r="E46" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="F46" s="4" t="s">
+      <c r="F46" s="11" t="s">
         <v>297</v>
       </c>
-      <c r="G46" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="H46" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="I46" s="2"/>
-      <c r="J46" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K46" s="2"/>
-      <c r="L46" s="2"/>
-      <c r="M46" s="2"/>
-      <c r="N46" s="2"/>
+      <c r="G46" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I46" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J46" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K46" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="L46" s="11" t="s">
+        <v>298</v>
+      </c>
+      <c r="M46" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="N46" s="10" t="s">
+        <v>299</v>
+      </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>39</v>
@@ -10883,19 +12245,19 @@
         <v>9</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>302</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="4" t="s">
@@ -10908,7 +12270,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>39</v>
@@ -10917,16 +12279,16 @@
         <v>9</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>84</v>
@@ -10940,78 +12302,74 @@
       <c r="M48" s="2"/>
       <c r="N48" s="2"/>
     </row>
-    <row r="49" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="10" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>26</v>
+        <v>39</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>308</v>
-      </c>
-      <c r="E49" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>311</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="G49" s="11" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="I49" s="10" t="s">
-        <v>74</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="I49" s="10"/>
       <c r="J49" s="11" t="s">
         <v>6</v>
       </c>
       <c r="K49" s="11" t="s">
-        <v>75</v>
+        <v>219</v>
       </c>
       <c r="L49" s="11" t="s">
-        <v>250</v>
+        <v>86</v>
       </c>
       <c r="M49" s="10" t="s">
-        <v>111</v>
+        <v>77</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>26</v>
+        <v>39</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="H50" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="I50" s="2" t="s">
-        <v>74</v>
-      </c>
+      <c r="I50" s="2"/>
       <c r="J50" s="4" t="s">
         <v>7</v>
       </c>
@@ -11022,186 +12380,194 @@
     </row>
     <row r="51" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="10" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>26</v>
+        <v>39</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="G51" s="11" t="s">
-        <v>20</v>
+        <v>83</v>
       </c>
       <c r="H51" s="10" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="11" t="s">
         <v>6</v>
       </c>
       <c r="K51" s="11" t="s">
-        <v>109</v>
+        <v>219</v>
       </c>
       <c r="L51" s="11" t="s">
-        <v>76</v>
+        <v>323</v>
       </c>
       <c r="M51" s="10" t="s">
-        <v>226</v>
+        <v>77</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D52" s="4" t="s">
+      <c r="A52" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" s="11" t="s">
+        <v>326</v>
+      </c>
+      <c r="E52" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="F52" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="G52" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="H52" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="I52" s="10"/>
+      <c r="J52" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K52" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="L52" s="11" t="s">
         <v>323</v>
       </c>
-      <c r="E52" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="F52" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="G52" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="I52" s="2"/>
-      <c r="J52" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K52" s="2"/>
-      <c r="L52" s="2"/>
-      <c r="M52" s="2"/>
-      <c r="N52" s="2"/>
+      <c r="M52" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="N52" s="10" t="s">
+        <v>329</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="B53" s="2" t="s">
+      <c r="A53" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="B53" s="10" t="s">
         <v>42</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D53" s="4" t="s">
-        <v>327</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="F53" s="4" t="s">
-        <v>329</v>
-      </c>
-      <c r="G53" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="I53" s="2"/>
-      <c r="J53" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K53" s="2"/>
-      <c r="L53" s="2"/>
-      <c r="M53" s="2"/>
-      <c r="N53" s="2"/>
+      <c r="D53" s="11" t="s">
+        <v>331</v>
+      </c>
+      <c r="E53" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="F53" s="11" t="s">
+        <v>333</v>
+      </c>
+      <c r="G53" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="H53" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I53" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J53" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K53" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="L53" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="M53" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="N53" s="10" t="s">
+        <v>335</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="10" t="s">
-        <v>330</v>
-      </c>
-      <c r="B54" s="10" t="s">
-        <v>46</v>
+      <c r="A54" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D54" s="11" t="s">
-        <v>331</v>
-      </c>
-      <c r="E54" s="11" t="s">
-        <v>332</v>
-      </c>
-      <c r="F54" s="11" t="s">
-        <v>333</v>
-      </c>
-      <c r="G54" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="H54" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="I54" s="10" t="s">
+      <c r="D54" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I54" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J54" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="K54" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="L54" s="11" t="s">
-        <v>334</v>
-      </c>
-      <c r="M54" s="10" t="s">
-        <v>220</v>
-      </c>
-      <c r="N54" s="10" t="s">
-        <v>335</v>
-      </c>
+      <c r="J54" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K54" s="2"/>
+      <c r="L54" s="2"/>
+      <c r="M54" s="2"/>
+      <c r="N54" s="2"/>
     </row>
     <row r="55" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="10" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>26</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="H55" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="I55" s="10" t="s">
-        <v>74</v>
-      </c>
+      <c r="I55" s="10"/>
       <c r="J55" s="11" t="s">
         <v>6</v>
       </c>
@@ -11209,36 +12575,36 @@
         <v>109</v>
       </c>
       <c r="L55" s="11" t="s">
-        <v>334</v>
+        <v>76</v>
       </c>
       <c r="M55" s="10" t="s">
         <v>220</v>
       </c>
       <c r="N55" s="10" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>48</v>
+        <v>201</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>73</v>
@@ -11254,25 +12620,25 @@
     </row>
     <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>26</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>84</v>
@@ -11287,60 +12653,70 @@
       <c r="N57" s="2"/>
     </row>
     <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="B58" s="2" t="s">
+      <c r="A58" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="B58" s="10" t="s">
         <v>46</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D58" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="E58" s="4" t="s">
-        <v>351</v>
-      </c>
-      <c r="F58" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="G58" s="4" t="s">
+      <c r="D58" s="11" t="s">
+        <v>354</v>
+      </c>
+      <c r="E58" s="11" t="s">
+        <v>355</v>
+      </c>
+      <c r="F58" s="11" t="s">
+        <v>356</v>
+      </c>
+      <c r="G58" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="H58" s="2" t="s">
+      <c r="H58" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="I58" s="2"/>
-      <c r="J58" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K58" s="2"/>
-      <c r="L58" s="2"/>
-      <c r="M58" s="2"/>
-      <c r="N58" s="2"/>
+      <c r="I58" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J58" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K58" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="L58" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="M58" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="N58" s="10" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="10" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>26</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="G59" s="11" t="s">
-        <v>357</v>
+        <v>48</v>
       </c>
       <c r="H59" s="10" t="s">
         <v>84</v>
@@ -11355,117 +12731,123 @@
         <v>109</v>
       </c>
       <c r="L59" s="11" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="M59" s="10" t="s">
-        <v>163</v>
+        <v>227</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="10" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="D60" s="11" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="G60" s="11" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="H60" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="I60" s="10" t="s">
-        <v>74</v>
-      </c>
+      <c r="I60" s="10"/>
       <c r="J60" s="11" t="s">
         <v>6</v>
       </c>
       <c r="K60" s="11" t="s">
-        <v>109</v>
+        <v>219</v>
       </c>
       <c r="L60" s="11" t="s">
-        <v>117</v>
+        <v>368</v>
       </c>
       <c r="M60" s="10" t="s">
-        <v>77</v>
+        <v>227</v>
       </c>
       <c r="N60" s="10" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2" t="s">
-        <v>365</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>50</v>
+      <c r="A61" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="B61" s="10" t="s">
+        <v>46</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D61" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="E61" s="4" t="s">
-        <v>367</v>
-      </c>
-      <c r="F61" s="4" t="s">
-        <v>368</v>
-      </c>
-      <c r="G61" s="4" t="s">
-        <v>369</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="I61" s="2"/>
-      <c r="J61" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K61" s="2"/>
-      <c r="L61" s="2"/>
-      <c r="M61" s="2"/>
-      <c r="N61" s="2"/>
+      <c r="D61" s="11" t="s">
+        <v>371</v>
+      </c>
+      <c r="E61" s="11" t="s">
+        <v>372</v>
+      </c>
+      <c r="F61" s="11" t="s">
+        <v>373</v>
+      </c>
+      <c r="G61" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="H61" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I61" s="10"/>
+      <c r="J61" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K61" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="L61" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="M61" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="N61" s="10" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>26</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>357</v>
+        <v>48</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I62" s="2"/>
       <c r="J62" s="4" t="s">
@@ -11476,8 +12858,290 @@
       <c r="M62" s="2"/>
       <c r="N62" s="2"/>
     </row>
+    <row r="63" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="10" t="s">
+        <v>379</v>
+      </c>
+      <c r="B63" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63" s="11" t="s">
+        <v>380</v>
+      </c>
+      <c r="E63" s="11" t="s">
+        <v>381</v>
+      </c>
+      <c r="F63" s="11" t="s">
+        <v>382</v>
+      </c>
+      <c r="G63" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="H63" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I63" s="10"/>
+      <c r="J63" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K63" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="L63" s="11" t="s">
+        <v>383</v>
+      </c>
+      <c r="M63" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="N63" s="10" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="10" t="s">
+        <v>385</v>
+      </c>
+      <c r="B64" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D64" s="11" t="s">
+        <v>386</v>
+      </c>
+      <c r="E64" s="10" t="s">
+        <v>387</v>
+      </c>
+      <c r="F64" s="11" t="s">
+        <v>388</v>
+      </c>
+      <c r="G64" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="H64" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I64" s="10"/>
+      <c r="J64" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K64" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="L64" s="11" t="s">
+        <v>368</v>
+      </c>
+      <c r="M64" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="N64" s="10" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="10" t="s">
+        <v>390</v>
+      </c>
+      <c r="B65" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D65" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="E65" s="11" t="s">
+        <v>392</v>
+      </c>
+      <c r="F65" s="11" t="s">
+        <v>393</v>
+      </c>
+      <c r="G65" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="H65" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I65" s="10"/>
+      <c r="J65" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K65" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="L65" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="M65" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="N65" s="10" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="B66" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D66" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="E66" s="11" t="s">
+        <v>397</v>
+      </c>
+      <c r="F66" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="G66" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="H66" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="I66" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J66" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K66" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="L66" s="11" t="s">
+        <v>383</v>
+      </c>
+      <c r="M66" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="N66" s="10" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="10" t="s">
+        <v>401</v>
+      </c>
+      <c r="B67" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D67" s="11" t="s">
+        <v>402</v>
+      </c>
+      <c r="E67" s="11" t="s">
+        <v>403</v>
+      </c>
+      <c r="F67" s="11" t="s">
+        <v>404</v>
+      </c>
+      <c r="G67" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="H67" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I67" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J67" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="K67" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="L67" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="M67" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="N67" s="10" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="G68" s="4" t="s">
+        <v>410</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I68" s="2"/>
+      <c r="J68" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K68" s="2"/>
+      <c r="L68" s="2"/>
+      <c r="M68" s="2"/>
+      <c r="N68" s="2"/>
+    </row>
+    <row r="69" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I69" s="2"/>
+      <c r="J69" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K69" s="2"/>
+      <c r="L69" s="2"/>
+      <c r="M69" s="2"/>
+      <c r="N69" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N62"/>
+  <autoFilter ref="A1:N69"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -11503,10 +13167,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>374</v>
+        <v>415</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>375</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11514,7 +13178,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>376</v>
+        <v>417</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11522,7 +13186,7 @@
         <v>61</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11530,7 +13194,7 @@
         <v>62</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>378</v>
+        <v>419</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11538,39 +13202,39 @@
         <v>63</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>379</v>
+        <v>420</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>380</v>
+        <v>421</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>381</v>
+        <v>422</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>382</v>
+        <v>423</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>383</v>
+        <v>424</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>384</v>
+        <v>425</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>385</v>
+        <v>426</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>386</v>
+        <v>427</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>387</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>

</xml_diff>